<commit_message>
docs: actualizar guias y trackers institucionales
</commit_message>
<xml_diff>
--- a/outputs/seguimiento-chat-20260809/Tracker_Seguimiento_Chat_LDSM.xlsx
+++ b/outputs/seguimiento-chat-20260809/Tracker_Seguimiento_Chat_LDSM.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="R7eac9d352e514af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" r:id="Rcc37e7980205442a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1104,20 +1104,20 @@
       </x:c>
       <x:c r="G6" s="28"/>
       <x:c r="H6" s="48" t="n">
-        <x:v>46243</x:v>
+        <x:v>46244</x:v>
       </x:c>
       <x:c r="I6" s="41"/>
       <x:c r="J6" s="15"/>
       <x:c r="K6" s="42" t="n">
         <x:f>COUNTA($C$10:$C$39)</x:f>
-        <x:v>28</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="L6" s="43"/>
       <x:c r="M6" s="43"/>
       <x:c r="N6" s="44"/>
       <x:c r="O6" s="45" t="n">
         <x:f>COUNTIF($E$10:$E$39,"Complete")</x:f>
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="P6" s="46"/>
       <x:c r="Q6" s="46"/>
@@ -1138,7 +1138,7 @@
       <x:c r="Z6" s="40"/>
       <x:c r="AA6" s="38" t="n">
         <x:f>COUNTIF($F$10:$F$39,"P0")</x:f>
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="AB6" s="39"/>
       <x:c r="AC6" s="39"/>
@@ -1290,11 +1290,11 @@
       <x:c r="J9" s="15"/>
       <x:c r="K9" s="2" t="n">
         <x:f>$H$6</x:f>
-        <x:v>46243</x:v>
+        <x:v>46244</x:v>
       </x:c>
       <x:c r="L9" s="2" t="n">
         <x:f t="shared" ref="L9:AD9" si="0">K9+7</x:f>
-        <x:v>46250</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="M9" s="2">
         <x:f t="shared" si="0"/>
@@ -1396,9 +1396,8 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J10" s="15"/>
-      <x:c r="K10" s="12" t="n">
+      <x:c r="K10" s="12" t="str">
         <x:f t="shared" ref="K10:T19" si="2">IF(OR($G10="",$H10="",$H10&lt;$G10),"",IF(AND(K$9&lt;=$H10,K$9+6&gt;=$G10),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="L10" s="13" t="str">
         <x:f t="shared" si="2">IF(OR($G10="",$H10="",$H10&lt;$G10),"",IF(AND(L$9&lt;=$H10,L$9+6&gt;=$G10),1,""))</x:f>
@@ -1486,9 +1485,8 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J11" s="15"/>
-      <x:c r="K11" s="12" t="n">
+      <x:c r="K11" s="12" t="str">
         <x:f t="shared" si="2">IF(OR($G11="",$H11="",$H11&lt;$G11),"",IF(AND(K$9&lt;=$H11,K$9+6&gt;=$G11),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="L11" s="13" t="str">
         <x:f t="shared" si="2">IF(OR($G11="",$H11="",$H11&lt;$G11),"",IF(AND(L$9&lt;=$H11,L$9+6&gt;=$G11),1,""))</x:f>
@@ -2366,7 +2364,7 @@
         <x:v>Seguimiento institucional</x:v>
       </x:c>
       <x:c r="C21" s="3" t="str">
-        <x:v>Pruebas unitarias, API, UI y regresión</x:v>
+        <x:v>Pruebas unitarias, API, UI y regresión completa con límite por cuenta e IP</x:v>
       </x:c>
       <x:c r="D21" s="8" t="str">
         <x:v>Codex (local)</x:v>
@@ -2568,9 +2566,8 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J23" s="15"/>
-      <x:c r="K23" s="12" t="n">
+      <x:c r="K23" s="12" t="str">
         <x:f t="shared" si="4">IF(OR($G23="",$H23="",$H23&lt;$G23),"",IF(AND(K$9&lt;=$H23,K$9+6&gt;=$G23),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="L23" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G23="",$H23="",$H23&lt;$G23),"",IF(AND(L$9&lt;=$H23,L$9+6&gt;=$G23),1,""))</x:f>
@@ -2658,9 +2655,8 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="J24" s="15"/>
-      <x:c r="K24" s="12" t="n">
+      <x:c r="K24" s="12" t="str">
         <x:f t="shared" si="4">IF(OR($G24="",$H24="",$H24&lt;$G24),"",IF(AND(K$9&lt;=$H24,K$9+6&gt;=$G24),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="L24" s="13" t="str">
         <x:f t="shared" si="4">IF(OR($G24="",$H24="",$H24&lt;$G24),"",IF(AND(L$9&lt;=$H24,L$9+6&gt;=$G24),1,""))</x:f>
@@ -3176,7 +3172,7 @@
         <x:v>Chat interno</x:v>
       </x:c>
       <x:c r="C30" s="4" t="str">
-        <x:v>Crear interfaz de conversaciones y mensajes</x:v>
+        <x:v>Actualizar mensajes en tiempo real con SSE y sondeo de respaldo</x:v>
       </x:c>
       <x:c r="D30" s="7" t="str">
         <x:v>Codex (local)</x:v>
@@ -3188,14 +3184,14 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G30" s="49" t="n">
-        <x:v>46247</x:v>
+        <x:v>46244</x:v>
       </x:c>
       <x:c r="H30" s="49" t="n">
-        <x:v>46249</x:v>
+        <x:v>46244</x:v>
       </x:c>
       <x:c r="I30" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G30="",H30="",H30&lt;G30),"",H30-G30+1)</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J30" s="15"/>
       <x:c r="K30" s="12" t="n">
@@ -3266,7 +3262,7 @@
         <x:v>Chat interno</x:v>
       </x:c>
       <x:c r="C31" s="3" t="str">
-        <x:v>Agregar buscador, estados vacíos y responsive móvil</x:v>
+        <x:v>Configurar retención global y por conversación con previsualización segura</x:v>
       </x:c>
       <x:c r="D31" s="8" t="str">
         <x:v>Codex (local)</x:v>
@@ -3275,17 +3271,17 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F31" s="8" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="G31" s="51" t="n">
-        <x:v>46248</x:v>
+        <x:v>46244</x:v>
       </x:c>
       <x:c r="H31" s="51" t="n">
-        <x:v>46249</x:v>
+        <x:v>46244</x:v>
       </x:c>
       <x:c r="I31" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G31="",H31="",H31&lt;G31),"",H31-G31+1)</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J31" s="15"/>
       <x:c r="K31" s="12" t="n">
@@ -3356,7 +3352,7 @@
         <x:v>Chat interno</x:v>
       </x:c>
       <x:c r="C32" s="4" t="str">
-        <x:v>Integrar indicador de no leídos, panel y ayuda</x:v>
+        <x:v>Crear interfaz de conversaciones y mensajes</x:v>
       </x:c>
       <x:c r="D32" s="7" t="str">
         <x:v>Codex (local)</x:v>
@@ -3365,26 +3361,25 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F32" s="7" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="G32" s="52" t="n">
+        <x:v>46247</x:v>
+      </x:c>
+      <x:c r="H32" s="52" t="n">
         <x:v>46249</x:v>
-      </x:c>
-      <x:c r="H32" s="52" t="n">
-        <x:v>46250</x:v>
       </x:c>
       <x:c r="I32" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G32="",H32="",H32&lt;G32),"",H32-G32+1)</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J32" s="15"/>
       <x:c r="K32" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G32="",$H32="",$H32&lt;$G32),"",IF(AND(K$9&lt;=$H32,K$9+6&gt;=$G32),1,""))</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L32" s="13" t="n">
+      <x:c r="L32" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G32="",$H32="",$H32&lt;$G32),"",IF(AND(L$9&lt;=$H32,L$9+6&gt;=$G32),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="M32" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G32="",$H32="",$H32&lt;$G32),"",IF(AND(M$9&lt;=$H32,M$9+6&gt;=$G32),1,""))</x:f>
@@ -3447,7 +3442,7 @@
         <x:v>Chat interno</x:v>
       </x:c>
       <x:c r="C33" s="3" t="str">
-        <x:v>Pruebas de aislamiento, permisos y regresión</x:v>
+        <x:v>Agregar buscador, estados vacíos y responsive móvil</x:v>
       </x:c>
       <x:c r="D33" s="8" t="str">
         <x:v>Codex (local)</x:v>
@@ -3456,25 +3451,25 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F33" s="8" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="G33" s="51" t="n">
-        <x:v>46250</x:v>
+        <x:v>46248</x:v>
       </x:c>
       <x:c r="H33" s="51" t="n">
-        <x:v>46251</x:v>
+        <x:v>46249</x:v>
       </x:c>
       <x:c r="I33" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G33="",H33="",H33&lt;G33),"",H33-G33+1)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J33" s="15"/>
-      <x:c r="K33" s="12" t="str">
+      <x:c r="K33" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(K$9&lt;=$H33,K$9+6&gt;=$G33),1,""))</x:f>
-      </x:c>
-      <x:c r="L33" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L33" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(L$9&lt;=$H33,L$9+6&gt;=$G33),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="M33" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(M$9&lt;=$H33,M$9+6&gt;=$G33),1,""))</x:f>
@@ -3489,9 +3484,8 @@
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(P$9&lt;=$H33,P$9+6&gt;=$G33),1,""))</x:f>
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q33" s="12" t="n">
+      <x:c r="Q33" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(Q$9&lt;=$H33,Q$9+6&gt;=$G33),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="R33" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G33="",$H33="",$H33&lt;$G33),"",IF(AND(R$9&lt;=$H33,R$9+6&gt;=$G33),1,""))</x:f>
@@ -3538,34 +3532,34 @@
         <x:v>Chat interno</x:v>
       </x:c>
       <x:c r="C34" s="4" t="str">
-        <x:v>Aprobar política institucional de retención y uso</x:v>
+        <x:v>Integrar indicador de no leídos, panel y ayuda</x:v>
       </x:c>
       <x:c r="D34" s="7" t="str">
-        <x:v>Equipo escolar</x:v>
+        <x:v>Codex (local)</x:v>
       </x:c>
       <x:c r="E34" s="7" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Complete</x:v>
       </x:c>
       <x:c r="F34" s="7" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="G34" s="52" t="n">
-        <x:v>46251</x:v>
+        <x:v>46249</x:v>
       </x:c>
       <x:c r="H34" s="52" t="n">
-        <x:v>46255</x:v>
+        <x:v>46250</x:v>
       </x:c>
       <x:c r="I34" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G34="",H34="",H34&lt;G34),"",H34-G34+1)</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J34" s="15"/>
-      <x:c r="K34" s="12" t="str">
+      <x:c r="K34" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(K$9&lt;=$H34,K$9+6&gt;=$G34),1,""))</x:f>
-      </x:c>
-      <x:c r="L34" s="13" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L34" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(L$9&lt;=$H34,L$9+6&gt;=$G34),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="M34" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(M$9&lt;=$H34,M$9+6&gt;=$G34),1,""))</x:f>
@@ -3576,12 +3570,12 @@
       <x:c r="O34" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(O$9&lt;=$H34,O$9+6&gt;=$G34),1,""))</x:f>
       </x:c>
-      <x:c r="P34" s="13" t="str">
+      <x:c r="P34" s="13" t="n">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(P$9&lt;=$H34,P$9+6&gt;=$G34),1,""))</x:f>
-      </x:c>
-      <x:c r="Q34" s="12" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="Q34" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(Q$9&lt;=$H34,Q$9+6&gt;=$G34),1,""))</x:f>
-        <x:v>1</x:v>
       </x:c>
       <x:c r="R34" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G34="",$H34="",$H34&lt;$G34),"",IF(AND(R$9&lt;=$H34,R$9+6&gt;=$G34),1,""))</x:f>
@@ -3625,10 +3619,10 @@
     </x:row>
     <x:row r="35">
       <x:c r="B35" s="6" t="str">
-        <x:v>Calidad transversal</x:v>
+        <x:v>Chat interno</x:v>
       </x:c>
       <x:c r="C35" s="3" t="str">
-        <x:v>Ejecutar lint, pruebas, build y migración aislada</x:v>
+        <x:v>Pruebas de aislamiento, permisos y regresión</x:v>
       </x:c>
       <x:c r="D35" s="8" t="str">
         <x:v>Codex (local)</x:v>
@@ -3640,18 +3634,19 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="G35" s="51" t="n">
+        <x:v>46250</x:v>
+      </x:c>
+      <x:c r="H35" s="51" t="n">
         <x:v>46251</x:v>
-      </x:c>
-      <x:c r="H35" s="51" t="n">
-        <x:v>46252</x:v>
       </x:c>
       <x:c r="I35" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G35="",H35="",H35&lt;G35),"",H35-G35+1)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="J35" s="15"/>
-      <x:c r="K35" s="12" t="str">
+      <x:c r="K35" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(K$9&lt;=$H35,K$9+6&gt;=$G35),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="L35" s="13" t="n">
         <x:f t="shared" si="6">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(L$9&lt;=$H35,L$9+6&gt;=$G35),1,""))</x:f>
@@ -3666,8 +3661,9 @@
       <x:c r="O35" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(O$9&lt;=$H35,O$9+6&gt;=$G35),1,""))</x:f>
       </x:c>
-      <x:c r="P35" s="13" t="str">
+      <x:c r="P35" s="13" t="n">
         <x:f t="shared" si="6">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(P$9&lt;=$H35,P$9+6&gt;=$G35),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="Q35" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G35="",$H35="",$H35&lt;$G35),"",IF(AND(Q$9&lt;=$H35,Q$9+6&gt;=$G35),1,""))</x:f>
@@ -3715,29 +3711,29 @@
     </x:row>
     <x:row r="36">
       <x:c r="B36" s="5" t="str">
-        <x:v>Calidad transversal</x:v>
+        <x:v>Chat interno</x:v>
       </x:c>
       <x:c r="C36" s="4" t="str">
-        <x:v>Auditar accesibilidad y experiencia móvil</x:v>
+        <x:v>Aprobar política institucional de retención y uso</x:v>
       </x:c>
       <x:c r="D36" s="7" t="str">
-        <x:v>Codex (local)</x:v>
+        <x:v>Equipo escolar</x:v>
       </x:c>
       <x:c r="E36" s="7" t="str">
-        <x:v>Complete</x:v>
+        <x:v>Not Started</x:v>
       </x:c>
       <x:c r="F36" s="7" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="G36" s="52" t="n">
-        <x:v>46252</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="H36" s="52" t="n">
-        <x:v>46253</x:v>
+        <x:v>46255</x:v>
       </x:c>
       <x:c r="I36" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G36="",H36="",H36&lt;G36),"",H36-G36+1)</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J36" s="15"/>
       <x:c r="K36" s="12" t="str">
@@ -3808,7 +3804,7 @@
         <x:v>Calidad transversal</x:v>
       </x:c>
       <x:c r="C37" s="3" t="str">
-        <x:v>Preparar evidencia y guía de pruebas</x:v>
+        <x:v>Ejecutar lint, pruebas, build y migración aislada</x:v>
       </x:c>
       <x:c r="D37" s="8" t="str">
         <x:v>Codex (local)</x:v>
@@ -3817,13 +3813,13 @@
         <x:v>Complete</x:v>
       </x:c>
       <x:c r="F37" s="8" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="G37" s="51" t="n">
-        <x:v>46253</x:v>
+        <x:v>46251</x:v>
       </x:c>
       <x:c r="H37" s="51" t="n">
-        <x:v>46254</x:v>
+        <x:v>46252</x:v>
       </x:c>
       <x:c r="I37" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G37="",H37="",H37&lt;G37),"",H37-G37+1)</x:f>
@@ -3894,22 +3890,38 @@
       </x:c>
     </x:row>
     <x:row r="38">
-      <x:c r="B38" s="5"/>
-      <x:c r="C38" s="4"/>
-      <x:c r="D38" s="7"/>
-      <x:c r="E38" s="7"/>
-      <x:c r="F38" s="7"/>
-      <x:c r="G38" s="9"/>
-      <x:c r="H38" s="9"/>
-      <x:c r="I38" s="11" t="str">
+      <x:c r="B38" s="5" t="str">
+        <x:v>Calidad transversal</x:v>
+      </x:c>
+      <x:c r="C38" s="4" t="str">
+        <x:v>Auditar accesibilidad y experiencia móvil</x:v>
+      </x:c>
+      <x:c r="D38" s="7" t="str">
+        <x:v>Codex (local)</x:v>
+      </x:c>
+      <x:c r="E38" s="7" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="F38" s="7" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="G38" s="52" t="n">
+        <x:v>46252</x:v>
+      </x:c>
+      <x:c r="H38" s="52" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="I38" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G38="",H38="",H38&lt;G38),"",H38-G38+1)</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J38" s="15"/>
       <x:c r="K38" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(K$9&lt;=$H38,K$9+6&gt;=$G38),1,""))</x:f>
       </x:c>
-      <x:c r="L38" s="13" t="str">
+      <x:c r="L38" s="13" t="n">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(L$9&lt;=$H38,L$9+6&gt;=$G38),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M38" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(M$9&lt;=$H38,M$9+6&gt;=$G38),1,""))</x:f>
@@ -3923,8 +3935,9 @@
       <x:c r="P38" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(P$9&lt;=$H38,P$9+6&gt;=$G38),1,""))</x:f>
       </x:c>
-      <x:c r="Q38" s="12" t="str">
+      <x:c r="Q38" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(Q$9&lt;=$H38,Q$9+6&gt;=$G38),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R38" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G38="",$H38="",$H38&lt;$G38),"",IF(AND(R$9&lt;=$H38,R$9+6&gt;=$G38),1,""))</x:f>
@@ -3967,22 +3980,38 @@
       </x:c>
     </x:row>
     <x:row r="39">
-      <x:c r="B39" s="6"/>
-      <x:c r="C39" s="3"/>
-      <x:c r="D39" s="8"/>
-      <x:c r="E39" s="8"/>
-      <x:c r="F39" s="8"/>
-      <x:c r="G39" s="10"/>
-      <x:c r="H39" s="10"/>
-      <x:c r="I39" s="11" t="str">
+      <x:c r="B39" s="6" t="str">
+        <x:v>Calidad transversal</x:v>
+      </x:c>
+      <x:c r="C39" s="3" t="str">
+        <x:v>Preparar evidencia y guía de pruebas</x:v>
+      </x:c>
+      <x:c r="D39" s="8" t="str">
+        <x:v>Codex (local)</x:v>
+      </x:c>
+      <x:c r="E39" s="8" t="str">
+        <x:v>Complete</x:v>
+      </x:c>
+      <x:c r="F39" s="8" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="G39" s="51" t="n">
+        <x:v>46253</x:v>
+      </x:c>
+      <x:c r="H39" s="51" t="n">
+        <x:v>46254</x:v>
+      </x:c>
+      <x:c r="I39" s="11" t="n">
         <x:f t="shared" si="1">IF(OR(G39="",H39="",H39&lt;G39),"",H39-G39+1)</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="J39" s="15"/>
       <x:c r="K39" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G39="",$H39="",$H39&lt;$G39),"",IF(AND(K$9&lt;=$H39,K$9+6&gt;=$G39),1,""))</x:f>
       </x:c>
-      <x:c r="L39" s="13" t="str">
+      <x:c r="L39" s="13" t="n">
         <x:f t="shared" si="6">IF(OR($G39="",$H39="",$H39&lt;$G39),"",IF(AND(L$9&lt;=$H39,L$9+6&gt;=$G39),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="M39" s="12" t="str">
         <x:f t="shared" si="6">IF(OR($G39="",$H39="",$H39&lt;$G39),"",IF(AND(M$9&lt;=$H39,M$9+6&gt;=$G39),1,""))</x:f>
@@ -3996,8 +4025,9 @@
       <x:c r="P39" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G39="",$H39="",$H39&lt;$G39),"",IF(AND(P$9&lt;=$H39,P$9+6&gt;=$G39),1,""))</x:f>
       </x:c>
-      <x:c r="Q39" s="12" t="str">
+      <x:c r="Q39" s="12" t="n">
         <x:f t="shared" si="6">IF(OR($G39="",$H39="",$H39&lt;$G39),"",IF(AND(Q$9&lt;=$H39,Q$9+6&gt;=$G39),1,""))</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="R39" s="13" t="str">
         <x:f t="shared" si="6">IF(OR($G39="",$H39="",$H39&lt;$G39),"",IF(AND(R$9&lt;=$H39,R$9+6&gt;=$G39),1,""))</x:f>
@@ -4072,7 +4102,7 @@
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="B41" s="29" t="str">
-        <x:v>Estado local al 09-08-2026: implementación y QA automatizada completas. Quedan únicamente la validación escolar de reglas automáticas y la aprobación institucional de retención del chat. La automatización permanece desactivada por defecto.</x:v>
+        <x:v>Estado local al 10-08-2026: implementación y QA automatizada completas. Seguimiento incorpora asignación, escalamiento y avisos; Chat incorpora tiempo real, silencios y retención configurable. La regresión final aprobó 143 pruebas backend, 47 frontend y 32 recorridos E2E; 2 casos se omitieron intencionalmente. Quedan la validación escolar de reglas y la aprobación institucional de retención. Ambas automatizaciones permanecen desactivadas por defecto.</x:v>
       </x:c>
       <x:c r="C41" s="30" t="str"/>
       <x:c r="D41" s="30" t="str"/>

</xml_diff>